<commit_message>
Update output/DMcard Wave Spreadsheet-WAVE Updated.xlsx via Generic Excel Template Updater
</commit_message>
<xml_diff>
--- a/output/DMcard Wave Spreadsheet-WAVE Updated.xlsx
+++ b/output/DMcard Wave Spreadsheet-WAVE Updated.xlsx
@@ -637,17 +637,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>03/05/2026</t>
+          <t>05/12/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Pacific Financial Services</t>
+          <t>United Regional Bank</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>503</t>
+          <t>505</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -677,29 +677,29 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>15600</t>
+          <t>19200</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>SMS, Mobile App</t>
+          <t>SMS</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>04/20/2026</t>
+          <t>06/01/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Metro Bank</t>
+          <t>Sunrise Financial</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>504</t>
+          <t>506</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -729,12 +729,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>6400</t>
+          <t>7300</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>IVR, SMS, Mobile App</t>
+          <t>IVR, Mobile App</t>
         </is>
       </c>
     </row>

</xml_diff>